<commit_message>
WIP: preserva continuación dos y controles pendientes
</commit_message>
<xml_diff>
--- a/tests/oracle/ORACULO_banca.xlsx
+++ b/tests/oracle/ORACULO_banca.xlsx
@@ -5384,242 +5384,242 @@
           <t>CONS-08</t>
         </is>
       </c>
-      <c r="FA1" t="inlineStr">
+      <c r="FA1" s="0" t="inlineStr">
         <is>
           <t>capitalInicial</t>
         </is>
       </c>
-      <c r="FB1" t="inlineStr">
+      <c r="FB1" s="0" t="inlineStr">
         <is>
           <t>compraActivos</t>
         </is>
       </c>
-      <c r="FC1" t="inlineStr">
+      <c r="FC1" s="0" t="inlineStr">
         <is>
           <t>adquisicionNeta</t>
         </is>
       </c>
-      <c r="FD1" t="inlineStr">
+      <c r="FD1" s="0" t="inlineStr">
         <is>
           <t>valorCompradoNeto</t>
         </is>
       </c>
-      <c r="FE1" t="inlineStr">
+      <c r="FE1" s="0" t="inlineStr">
         <is>
           <t>valorInventarioNeto</t>
         </is>
       </c>
-      <c r="FF1" t="inlineStr">
+      <c r="FF1" s="0" t="inlineStr">
         <is>
           <t>cajaInicial</t>
         </is>
       </c>
-      <c r="FG1" t="inlineStr">
+      <c r="FG1" s="0" t="inlineStr">
         <is>
           <t>tasaNuevoPrestamo</t>
         </is>
       </c>
-      <c r="FH1" t="inlineStr">
+      <c r="FH1" s="0" t="inlineStr">
         <is>
           <t>interesMensual</t>
         </is>
       </c>
-      <c r="FI1" t="inlineStr">
+      <c r="FI1" s="0" t="inlineStr">
         <is>
           <t>tasaMensual</t>
         </is>
       </c>
-      <c r="FJ1" t="inlineStr">
+      <c r="FJ1" s="0" t="inlineStr">
         <is>
           <t>intereses</t>
         </is>
       </c>
-      <c r="FK1" t="inlineStr">
+      <c r="FK1" s="0" t="inlineStr">
         <is>
           <t>pagosOperacion</t>
         </is>
       </c>
-      <c r="FL1" t="inlineStr">
+      <c r="FL1" s="0" t="inlineStr">
         <is>
           <t>cajaFinal</t>
         </is>
       </c>
-      <c r="FM1" t="inlineStr">
+      <c r="FM1" s="0" t="inlineStr">
         <is>
           <t>depreciacionAcumulada</t>
         </is>
       </c>
-      <c r="FN1" t="inlineStr">
+      <c r="FN1" s="0" t="inlineStr">
         <is>
           <t>activosCosto</t>
         </is>
       </c>
-      <c r="FO1" t="inlineStr">
+      <c r="FO1" s="0" t="inlineStr">
         <is>
           <t>activosFijos</t>
         </is>
       </c>
-      <c r="FP1" t="inlineStr">
+      <c r="FP1" s="0" t="inlineStr">
         <is>
           <t>financial.estadoResultados.ingresos</t>
         </is>
       </c>
-      <c r="FQ1" t="inlineStr">
+      <c r="FQ1" s="0" t="inlineStr">
         <is>
           <t>financial.estadoResultados.ventasNetas</t>
         </is>
       </c>
-      <c r="FR1" t="inlineStr">
+      <c r="FR1" s="0" t="inlineStr">
         <is>
           <t>financial.estadoResultados.costos</t>
         </is>
       </c>
-      <c r="FS1" t="inlineStr">
+      <c r="FS1" s="0" t="inlineStr">
         <is>
           <t>financial.estadoResultados.utilidad</t>
         </is>
       </c>
-      <c r="FT1" t="inlineStr">
+      <c r="FT1" s="0" t="inlineStr">
         <is>
           <t>financial.estadoResultados.depreciacion</t>
         </is>
       </c>
-      <c r="FU1" t="inlineStr">
+      <c r="FU1" s="0" t="inlineStr">
         <is>
           <t>financial.estadoResultados.intereses</t>
         </is>
       </c>
-      <c r="FV1" t="inlineStr">
+      <c r="FV1" s="0" t="inlineStr">
         <is>
           <t>financial.estadoResultados.costosProduccion</t>
         </is>
       </c>
-      <c r="FW1" t="inlineStr">
+      <c r="FW1" s="0" t="inlineStr">
         <is>
           <t>financial.balanceCaja.cajaInicial</t>
         </is>
       </c>
-      <c r="FX1" t="inlineStr">
+      <c r="FX1" s="0" t="inlineStr">
         <is>
           <t>financial.balanceCaja.entradas</t>
         </is>
       </c>
-      <c r="FY1" t="inlineStr">
+      <c r="FY1" s="0" t="inlineStr">
         <is>
           <t>financial.balanceCaja.salidas</t>
         </is>
       </c>
-      <c r="FZ1" t="inlineStr">
+      <c r="FZ1" s="0" t="inlineStr">
         <is>
           <t>financial.balanceCaja.cajaFinal</t>
         </is>
       </c>
-      <c r="GA1" t="inlineStr">
+      <c r="GA1" s="0" t="inlineStr">
         <is>
           <t>financial.flujoCaja.cajaInicial</t>
         </is>
       </c>
-      <c r="GB1" t="inlineStr">
+      <c r="GB1" s="0" t="inlineStr">
         <is>
           <t>financial.flujoCaja.cobrosVentas</t>
         </is>
       </c>
-      <c r="GC1" t="inlineStr">
+      <c r="GC1" s="0" t="inlineStr">
         <is>
           <t>financial.flujoCaja.pagosOperacion</t>
         </is>
       </c>
-      <c r="GD1" t="inlineStr">
+      <c r="GD1" s="0" t="inlineStr">
         <is>
           <t>financial.flujoCaja.compraActivos</t>
         </is>
       </c>
-      <c r="GE1" t="inlineStr">
+      <c r="GE1" s="0" t="inlineStr">
         <is>
           <t>financial.flujoCaja.financiamiento</t>
         </is>
       </c>
-      <c r="GF1" t="inlineStr">
+      <c r="GF1" s="0" t="inlineStr">
         <is>
           <t>financial.flujoCaja.operacion</t>
         </is>
       </c>
-      <c r="GG1" t="inlineStr">
+      <c r="GG1" s="0" t="inlineStr">
         <is>
           <t>financial.flujoCaja.inversion</t>
         </is>
       </c>
-      <c r="GH1" t="inlineStr">
+      <c r="GH1" s="0" t="inlineStr">
         <is>
           <t>financial.flujoCaja.flujoNeto</t>
         </is>
       </c>
-      <c r="GI1" t="inlineStr">
+      <c r="GI1" s="0" t="inlineStr">
         <is>
           <t>financial.flujoCaja.cajaFinal</t>
         </is>
       </c>
-      <c r="GJ1" t="inlineStr">
+      <c r="GJ1" s="0" t="inlineStr">
         <is>
           <t>financial.balanceGeneral.efectivo</t>
         </is>
       </c>
-      <c r="GK1" t="inlineStr">
+      <c r="GK1" s="0" t="inlineStr">
         <is>
           <t>financial.balanceGeneral.activosFijos</t>
         </is>
       </c>
-      <c r="GL1" t="inlineStr">
+      <c r="GL1" s="0" t="inlineStr">
         <is>
           <t>financial.balanceGeneral.inventarioMP</t>
         </is>
       </c>
-      <c r="GM1" t="inlineStr">
+      <c r="GM1" s="0" t="inlineStr">
         <is>
           <t>financial.balanceGeneral.activos</t>
         </is>
       </c>
-      <c r="GN1" t="inlineStr">
+      <c r="GN1" s="0" t="inlineStr">
         <is>
           <t>financial.balanceGeneral.deuda</t>
         </is>
       </c>
-      <c r="GO1" t="inlineStr">
+      <c r="GO1" s="0" t="inlineStr">
         <is>
           <t>financial.balanceGeneral.patrimonio</t>
         </is>
       </c>
-      <c r="GP1" t="inlineStr">
+      <c r="GP1" s="0" t="inlineStr">
         <is>
           <t>financial.balanceGeneral.pasivoPatrimonio</t>
         </is>
       </c>
-      <c r="GQ1" t="inlineStr">
+      <c r="GQ1" s="0" t="inlineStr">
         <is>
           <t>financial.financiamiento.montoPrestamo</t>
         </is>
       </c>
-      <c r="GR1" t="inlineStr">
+      <c r="GR1" s="0" t="inlineStr">
         <is>
           <t>financial.financiamiento.tasaTEA</t>
         </is>
       </c>
-      <c r="GS1" t="inlineStr">
+      <c r="GS1" s="0" t="inlineStr">
         <is>
           <t>financial.financiamiento.deudaPrincipal</t>
         </is>
       </c>
-      <c r="GT1" t="inlineStr">
+      <c r="GT1" s="0" t="inlineStr">
         <is>
           <t>financial.financiamiento.tasaAdicionalProximoPrestamo</t>
         </is>
       </c>
-      <c r="GU1" t="inlineStr">
+      <c r="GU1" s="0" t="inlineStr">
         <is>
           <t>financial.financiamiento.tasaMensual</t>
         </is>
       </c>
-      <c r="GV1" t="inlineStr">
+      <c r="GV1" s="0" t="inlineStr">
         <is>
           <t>financial.financiamiento.intereses</t>
         </is>
@@ -6172,194 +6172,194 @@
         <f>AND(K2=0,AF2&lt;5)</f>
         <v/>
       </c>
-      <c r="FA2" t="n">
+      <c r="FA2" s="0" t="n">
         <v>1000000</v>
       </c>
-      <c r="FB2">
+      <c r="FB2" s="0">
         <f>1*2500*(1+0.03+0.02)+1*3500*(1+0.03+0.02)+1*1200*(1+0.03+0.02)+1*300*(1+0+0.01)</f>
         <v/>
       </c>
-      <c r="FC2">
+      <c r="FC2" s="0">
         <f>1*2500+1*3500+1*1200+1*300</f>
         <v/>
       </c>
-      <c r="FD2">
+      <c r="FD2" s="0">
         <f>(CF2*25+CH2*45+CJ2*80+CL2*4+CN2*9+CP2*2+CR2*4+CT2*7)*0.8924</f>
         <v/>
       </c>
-      <c r="FE2">
+      <c r="FE2" s="0">
         <f>(DC2*25+DE2*45+DG2*80+DJ2*4+DL2*9+DO2*2+DQ2*4+DS2*7)*0.8924</f>
         <v/>
       </c>
-      <c r="FF2">
+      <c r="FF2" s="0">
         <f>FA2</f>
         <v/>
       </c>
-      <c r="FG2">
+      <c r="FG2" s="0">
         <f>(1+AR2/100)^(1/12)-1</f>
         <v/>
       </c>
-      <c r="FH2">
+      <c r="FH2" s="0">
         <f>0*0+AP2*FG2</f>
         <v/>
       </c>
-      <c r="FI2">
+      <c r="FI2" s="0">
         <f>IFERROR(FH2/(0+AP2),0)</f>
         <v/>
       </c>
-      <c r="FJ2">
+      <c r="FJ2" s="0">
         <f>FH2*1</f>
         <v/>
       </c>
-      <c r="FK2">
+      <c r="FK2" s="0">
         <f>EQ2-DW2-DU2+FD2+FJ2</f>
         <v/>
       </c>
-      <c r="FL2">
+      <c r="FL2" s="0">
         <f>FF2+EK2+AP2-FK2-FB2</f>
         <v/>
       </c>
-      <c r="FM2">
+      <c r="FM2" s="0">
         <f>0+DW2</f>
         <v/>
       </c>
-      <c r="FN2">
+      <c r="FN2" s="0">
         <f>0+FC2</f>
         <v/>
       </c>
-      <c r="FO2">
+      <c r="FO2" s="0">
         <f>FN2-FM2</f>
         <v/>
       </c>
-      <c r="FP2">
+      <c r="FP2" s="0">
         <f>EK2</f>
         <v/>
       </c>
-      <c r="FQ2">
+      <c r="FQ2" s="0">
         <f>EK2</f>
         <v/>
       </c>
-      <c r="FR2">
+      <c r="FR2" s="0">
         <f>EQ2+FJ2</f>
         <v/>
       </c>
-      <c r="FS2">
+      <c r="FS2" s="0">
         <f>ER2-FJ2</f>
         <v/>
       </c>
-      <c r="FT2">
+      <c r="FT2" s="0">
         <f>DW2</f>
         <v/>
       </c>
-      <c r="FU2">
+      <c r="FU2" s="0">
         <f>FJ2</f>
         <v/>
       </c>
-      <c r="FV2">
+      <c r="FV2" s="0">
         <f>EQ2</f>
         <v/>
       </c>
-      <c r="FW2">
+      <c r="FW2" s="0">
         <f>FF2</f>
         <v/>
       </c>
-      <c r="FX2">
+      <c r="FX2" s="0">
         <f>EK2+AP2</f>
         <v/>
       </c>
-      <c r="FY2">
+      <c r="FY2" s="0">
         <f>FK2+FB2</f>
         <v/>
       </c>
-      <c r="FZ2">
+      <c r="FZ2" s="0">
         <f>FL2</f>
         <v/>
       </c>
-      <c r="GA2">
+      <c r="GA2" s="0">
         <f>FF2</f>
         <v/>
       </c>
-      <c r="GB2">
+      <c r="GB2" s="0">
         <f>EK2</f>
         <v/>
       </c>
-      <c r="GC2">
+      <c r="GC2" s="0">
         <f>FK2</f>
         <v/>
       </c>
-      <c r="GD2">
+      <c r="GD2" s="0">
         <f>FB2</f>
         <v/>
       </c>
-      <c r="GE2">
+      <c r="GE2" s="0">
         <f>AP2</f>
         <v/>
       </c>
-      <c r="GF2">
+      <c r="GF2" s="0">
         <f>EK2-FK2</f>
         <v/>
       </c>
-      <c r="GG2">
+      <c r="GG2" s="0">
         <f>-FB2</f>
         <v/>
       </c>
-      <c r="GH2">
+      <c r="GH2" s="0">
         <f>FL2-FF2</f>
         <v/>
       </c>
-      <c r="GI2">
+      <c r="GI2" s="0">
         <f>FL2</f>
         <v/>
       </c>
-      <c r="GJ2">
+      <c r="GJ2" s="0">
         <f>FL2</f>
         <v/>
       </c>
-      <c r="GK2">
+      <c r="GK2" s="0">
         <f>FO2</f>
         <v/>
       </c>
-      <c r="GL2">
+      <c r="GL2" s="0">
         <f>FE2</f>
         <v/>
       </c>
-      <c r="GM2">
+      <c r="GM2" s="0">
         <f>FL2+FO2+FE2</f>
         <v/>
       </c>
-      <c r="GN2">
+      <c r="GN2" s="0">
         <f>AS2</f>
         <v/>
       </c>
-      <c r="GO2">
+      <c r="GO2" s="0">
         <f>FL2+FO2+FE2-AS2</f>
         <v/>
       </c>
-      <c r="GP2">
+      <c r="GP2" s="0">
         <f>FL2+FO2+FE2</f>
         <v/>
       </c>
-      <c r="GQ2">
+      <c r="GQ2" s="0">
         <f>AP2</f>
         <v/>
       </c>
-      <c r="GR2">
+      <c r="GR2" s="0">
         <f>AR2</f>
         <v/>
       </c>
-      <c r="GS2">
+      <c r="GS2" s="0">
         <f>AS2</f>
         <v/>
       </c>
-      <c r="GT2">
+      <c r="GT2" s="0">
         <f>AT2</f>
         <v/>
       </c>
-      <c r="GU2">
+      <c r="GU2" s="0">
         <f>FI2</f>
         <v/>
       </c>
-      <c r="GV2">
+      <c r="GV2" s="0">
         <f>FJ2</f>
         <v/>
       </c>
@@ -6939,194 +6939,194 @@
         <f>AND(K3=0,AF3&lt;5)</f>
         <v/>
       </c>
-      <c r="FA3" t="n">
+      <c r="FA3" s="0" t="n">
         <v>1000000</v>
       </c>
-      <c r="FB3">
+      <c r="FB3" s="0">
         <f>0*2500*(1+0.03+0.02)+0*3500*(1+0.03+0.02)+0*1200*(1+0.03+0.02)+0*300*(1+0+0.01)</f>
         <v/>
       </c>
-      <c r="FC3">
+      <c r="FC3" s="0">
         <f>0*2500+0*3500+0*1200+0*300</f>
         <v/>
       </c>
-      <c r="FD3">
+      <c r="FD3" s="0">
         <f>(CF3*25+CH3*45+CJ3*80+CL3*4+CN3*9+CP3*2+CR3*4+CT3*7)*0.9016000000000001</f>
         <v/>
       </c>
-      <c r="FE3">
+      <c r="FE3" s="0">
         <f>(DC3*25+DE3*45+DG3*80+DJ3*4+DL3*9+DO3*2+DQ3*4+DS3*7)*0.9016000000000001</f>
         <v/>
       </c>
-      <c r="FF3">
+      <c r="FF3" s="0">
         <f>FL2</f>
         <v/>
       </c>
-      <c r="FG3">
+      <c r="FG3" s="0">
         <f>(1+AR3/100)^(1/12)-1</f>
         <v/>
       </c>
-      <c r="FH3">
+      <c r="FH3" s="0">
         <f>AS2*FI2+AP3*FG3</f>
         <v/>
       </c>
-      <c r="FI3">
+      <c r="FI3" s="0">
         <f>IFERROR(FH3/(AS2+AP3),0)</f>
         <v/>
       </c>
-      <c r="FJ3">
+      <c r="FJ3" s="0">
         <f>FH3*1</f>
         <v/>
       </c>
-      <c r="FK3">
+      <c r="FK3" s="0">
         <f>EQ3-DW3-DU3+FD3+FJ3</f>
         <v/>
       </c>
-      <c r="FL3">
+      <c r="FL3" s="0">
         <f>FF3+EK3+AP3-FK3-FB3</f>
         <v/>
       </c>
-      <c r="FM3">
+      <c r="FM3" s="0">
         <f>FM2+DW3</f>
         <v/>
       </c>
-      <c r="FN3">
+      <c r="FN3" s="0">
         <f>FN2+FC3</f>
         <v/>
       </c>
-      <c r="FO3">
+      <c r="FO3" s="0">
         <f>FN3-FM3</f>
         <v/>
       </c>
-      <c r="FP3">
+      <c r="FP3" s="0">
         <f>EK3</f>
         <v/>
       </c>
-      <c r="FQ3">
+      <c r="FQ3" s="0">
         <f>EK3</f>
         <v/>
       </c>
-      <c r="FR3">
+      <c r="FR3" s="0">
         <f>EQ3+FJ3</f>
         <v/>
       </c>
-      <c r="FS3">
+      <c r="FS3" s="0">
         <f>ER3-FJ3</f>
         <v/>
       </c>
-      <c r="FT3">
+      <c r="FT3" s="0">
         <f>DW3</f>
         <v/>
       </c>
-      <c r="FU3">
+      <c r="FU3" s="0">
         <f>FJ3</f>
         <v/>
       </c>
-      <c r="FV3">
+      <c r="FV3" s="0">
         <f>EQ3</f>
         <v/>
       </c>
-      <c r="FW3">
+      <c r="FW3" s="0">
         <f>FF3</f>
         <v/>
       </c>
-      <c r="FX3">
+      <c r="FX3" s="0">
         <f>EK3+AP3</f>
         <v/>
       </c>
-      <c r="FY3">
+      <c r="FY3" s="0">
         <f>FK3+FB3</f>
         <v/>
       </c>
-      <c r="FZ3">
+      <c r="FZ3" s="0">
         <f>FL3</f>
         <v/>
       </c>
-      <c r="GA3">
+      <c r="GA3" s="0">
         <f>FF3</f>
         <v/>
       </c>
-      <c r="GB3">
+      <c r="GB3" s="0">
         <f>EK3</f>
         <v/>
       </c>
-      <c r="GC3">
+      <c r="GC3" s="0">
         <f>FK3</f>
         <v/>
       </c>
-      <c r="GD3">
+      <c r="GD3" s="0">
         <f>FB3</f>
         <v/>
       </c>
-      <c r="GE3">
+      <c r="GE3" s="0">
         <f>AP3</f>
         <v/>
       </c>
-      <c r="GF3">
+      <c r="GF3" s="0">
         <f>EK3-FK3</f>
         <v/>
       </c>
-      <c r="GG3">
+      <c r="GG3" s="0">
         <f>-FB3</f>
         <v/>
       </c>
-      <c r="GH3">
+      <c r="GH3" s="0">
         <f>FL3-FF3</f>
         <v/>
       </c>
-      <c r="GI3">
+      <c r="GI3" s="0">
         <f>FL3</f>
         <v/>
       </c>
-      <c r="GJ3">
+      <c r="GJ3" s="0">
         <f>FL3</f>
         <v/>
       </c>
-      <c r="GK3">
+      <c r="GK3" s="0">
         <f>FO3</f>
         <v/>
       </c>
-      <c r="GL3">
+      <c r="GL3" s="0">
         <f>FE3</f>
         <v/>
       </c>
-      <c r="GM3">
+      <c r="GM3" s="0">
         <f>FL3+FO3+FE3</f>
         <v/>
       </c>
-      <c r="GN3">
+      <c r="GN3" s="0">
         <f>AS3</f>
         <v/>
       </c>
-      <c r="GO3">
+      <c r="GO3" s="0">
         <f>FL3+FO3+FE3-AS3</f>
         <v/>
       </c>
-      <c r="GP3">
+      <c r="GP3" s="0">
         <f>FL3+FO3+FE3</f>
         <v/>
       </c>
-      <c r="GQ3">
+      <c r="GQ3" s="0">
         <f>AP3</f>
         <v/>
       </c>
-      <c r="GR3">
+      <c r="GR3" s="0">
         <f>AR3</f>
         <v/>
       </c>
-      <c r="GS3">
+      <c r="GS3" s="0">
         <f>AS3</f>
         <v/>
       </c>
-      <c r="GT3">
+      <c r="GT3" s="0">
         <f>AT3</f>
         <v/>
       </c>
-      <c r="GU3">
+      <c r="GU3" s="0">
         <f>FI3</f>
         <v/>
       </c>
-      <c r="GV3">
+      <c r="GV3" s="0">
         <f>FJ3</f>
         <v/>
       </c>
@@ -7706,194 +7706,194 @@
         <f>AND(K4=0,AF4&lt;5)</f>
         <v/>
       </c>
-      <c r="FA4" t="n">
+      <c r="FA4" s="0" t="n">
         <v>1000000</v>
       </c>
-      <c r="FB4">
+      <c r="FB4" s="0">
         <f>0*2500*(1+0.03+0.02)+0*3500*(1+0.03+0.02)+0*1200*(1+0.03+0.02)+0*300*(1+0+0.01)</f>
         <v/>
       </c>
-      <c r="FC4">
+      <c r="FC4" s="0">
         <f>0*2500+0*3500+0*1200+0*300</f>
         <v/>
       </c>
-      <c r="FD4">
+      <c r="FD4" s="0">
         <f>(CF4*25+CH4*45+CJ4*80+CL4*4+CN4*9+CP4*2+CR4*4+CT4*7)*0.9016000000000001</f>
         <v/>
       </c>
-      <c r="FE4">
+      <c r="FE4" s="0">
         <f>(DC4*25+DE4*45+DG4*80+DJ4*4+DL4*9+DO4*2+DQ4*4+DS4*7)*0.9016000000000001</f>
         <v/>
       </c>
-      <c r="FF4">
+      <c r="FF4" s="0">
         <f>FL3</f>
         <v/>
       </c>
-      <c r="FG4">
+      <c r="FG4" s="0">
         <f>(1+AR4/100)^(1/12)-1</f>
         <v/>
       </c>
-      <c r="FH4">
+      <c r="FH4" s="0">
         <f>AS3*FI3+AP4*FG4</f>
         <v/>
       </c>
-      <c r="FI4">
+      <c r="FI4" s="0">
         <f>IFERROR(FH4/(AS3+AP4),0)</f>
         <v/>
       </c>
-      <c r="FJ4">
+      <c r="FJ4" s="0">
         <f>FH4*1</f>
         <v/>
       </c>
-      <c r="FK4">
+      <c r="FK4" s="0">
         <f>EQ4-DW4-DU4+FD4+FJ4</f>
         <v/>
       </c>
-      <c r="FL4">
+      <c r="FL4" s="0">
         <f>FF4+EK4+AP4-FK4-FB4</f>
         <v/>
       </c>
-      <c r="FM4">
+      <c r="FM4" s="0">
         <f>FM3+DW4</f>
         <v/>
       </c>
-      <c r="FN4">
+      <c r="FN4" s="0">
         <f>FN3+FC4</f>
         <v/>
       </c>
-      <c r="FO4">
+      <c r="FO4" s="0">
         <f>FN4-FM4</f>
         <v/>
       </c>
-      <c r="FP4">
+      <c r="FP4" s="0">
         <f>EK4</f>
         <v/>
       </c>
-      <c r="FQ4">
+      <c r="FQ4" s="0">
         <f>EK4</f>
         <v/>
       </c>
-      <c r="FR4">
+      <c r="FR4" s="0">
         <f>EQ4+FJ4</f>
         <v/>
       </c>
-      <c r="FS4">
+      <c r="FS4" s="0">
         <f>ER4-FJ4</f>
         <v/>
       </c>
-      <c r="FT4">
+      <c r="FT4" s="0">
         <f>DW4</f>
         <v/>
       </c>
-      <c r="FU4">
+      <c r="FU4" s="0">
         <f>FJ4</f>
         <v/>
       </c>
-      <c r="FV4">
+      <c r="FV4" s="0">
         <f>EQ4</f>
         <v/>
       </c>
-      <c r="FW4">
+      <c r="FW4" s="0">
         <f>FF4</f>
         <v/>
       </c>
-      <c r="FX4">
+      <c r="FX4" s="0">
         <f>EK4+AP4</f>
         <v/>
       </c>
-      <c r="FY4">
+      <c r="FY4" s="0">
         <f>FK4+FB4</f>
         <v/>
       </c>
-      <c r="FZ4">
+      <c r="FZ4" s="0">
         <f>FL4</f>
         <v/>
       </c>
-      <c r="GA4">
+      <c r="GA4" s="0">
         <f>FF4</f>
         <v/>
       </c>
-      <c r="GB4">
+      <c r="GB4" s="0">
         <f>EK4</f>
         <v/>
       </c>
-      <c r="GC4">
+      <c r="GC4" s="0">
         <f>FK4</f>
         <v/>
       </c>
-      <c r="GD4">
+      <c r="GD4" s="0">
         <f>FB4</f>
         <v/>
       </c>
-      <c r="GE4">
+      <c r="GE4" s="0">
         <f>AP4</f>
         <v/>
       </c>
-      <c r="GF4">
+      <c r="GF4" s="0">
         <f>EK4-FK4</f>
         <v/>
       </c>
-      <c r="GG4">
+      <c r="GG4" s="0">
         <f>-FB4</f>
         <v/>
       </c>
-      <c r="GH4">
+      <c r="GH4" s="0">
         <f>FL4-FF4</f>
         <v/>
       </c>
-      <c r="GI4">
+      <c r="GI4" s="0">
         <f>FL4</f>
         <v/>
       </c>
-      <c r="GJ4">
+      <c r="GJ4" s="0">
         <f>FL4</f>
         <v/>
       </c>
-      <c r="GK4">
+      <c r="GK4" s="0">
         <f>FO4</f>
         <v/>
       </c>
-      <c r="GL4">
+      <c r="GL4" s="0">
         <f>FE4</f>
         <v/>
       </c>
-      <c r="GM4">
+      <c r="GM4" s="0">
         <f>FL4+FO4+FE4</f>
         <v/>
       </c>
-      <c r="GN4">
+      <c r="GN4" s="0">
         <f>AS4</f>
         <v/>
       </c>
-      <c r="GO4">
+      <c r="GO4" s="0">
         <f>FL4+FO4+FE4-AS4</f>
         <v/>
       </c>
-      <c r="GP4">
+      <c r="GP4" s="0">
         <f>FL4+FO4+FE4</f>
         <v/>
       </c>
-      <c r="GQ4">
+      <c r="GQ4" s="0">
         <f>AP4</f>
         <v/>
       </c>
-      <c r="GR4">
+      <c r="GR4" s="0">
         <f>AR4</f>
         <v/>
       </c>
-      <c r="GS4">
+      <c r="GS4" s="0">
         <f>AS4</f>
         <v/>
       </c>
-      <c r="GT4">
+      <c r="GT4" s="0">
         <f>AT4</f>
         <v/>
       </c>
-      <c r="GU4">
+      <c r="GU4" s="0">
         <f>FI4</f>
         <v/>
       </c>
-      <c r="GV4">
+      <c r="GV4" s="0">
         <f>FJ4</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
fix: alinea resumen y oráculo con las decisiones congeladas
</commit_message>
<xml_diff>
--- a/tests/oracle/ORACULO_banca.xlsx
+++ b/tests/oracle/ORACULO_banca.xlsx
@@ -4442,7 +4442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:GV4"/>
+  <dimension ref="A1:GW4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" style="184" min="1" max="1"/>
@@ -4601,6 +4601,7 @@
     <col width="20" customWidth="1" style="184" min="154" max="154"/>
     <col width="20" customWidth="1" style="184" min="155" max="155"/>
     <col width="20" customWidth="1" style="184" min="156" max="156"/>
+    <col width="20" customWidth="1" style="184" min="157" max="157"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5336,290 +5337,295 @@
       </c>
       <c r="EQ1" s="0" t="inlineStr">
         <is>
+          <t>costoAnalista</t>
+        </is>
+      </c>
+      <c r="ER1" s="0" t="inlineStr">
+        <is>
           <t>costosTotales</t>
         </is>
       </c>
-      <c r="ER1" s="0" t="inlineStr">
+      <c r="ES1" s="0" t="inlineStr">
         <is>
           <t>utilidad</t>
         </is>
       </c>
-      <c r="ES1" s="0" t="inlineStr">
+      <c r="ET1" s="0" t="inlineStr">
         <is>
           <t>CONS-01</t>
         </is>
       </c>
-      <c r="ET1" s="0" t="inlineStr">
+      <c r="EU1" s="0" t="inlineStr">
         <is>
           <t>CONS-02</t>
         </is>
       </c>
-      <c r="EU1" s="0" t="inlineStr">
+      <c r="EV1" s="0" t="inlineStr">
         <is>
           <t>CONS-03</t>
         </is>
       </c>
-      <c r="EV1" s="0" t="inlineStr">
+      <c r="EW1" s="0" t="inlineStr">
         <is>
           <t>CONS-04</t>
         </is>
       </c>
-      <c r="EW1" s="0" t="inlineStr">
+      <c r="EX1" s="0" t="inlineStr">
         <is>
           <t>CONS-05</t>
         </is>
       </c>
-      <c r="EX1" s="0" t="inlineStr">
+      <c r="EY1" s="0" t="inlineStr">
         <is>
           <t>CONS-06</t>
         </is>
       </c>
-      <c r="EY1" s="0" t="inlineStr">
+      <c r="EZ1" s="0" t="inlineStr">
         <is>
           <t>CONS-07</t>
         </is>
       </c>
-      <c r="EZ1" s="0" t="inlineStr">
+      <c r="FA1" s="0" t="inlineStr">
         <is>
           <t>CONS-08</t>
         </is>
       </c>
-      <c r="FA1" s="0" t="inlineStr">
+      <c r="FB1" t="inlineStr">
         <is>
           <t>capitalInicial</t>
         </is>
       </c>
-      <c r="FB1" s="0" t="inlineStr">
+      <c r="FC1" t="inlineStr">
         <is>
           <t>compraActivos</t>
         </is>
       </c>
-      <c r="FC1" s="0" t="inlineStr">
+      <c r="FD1" t="inlineStr">
         <is>
           <t>adquisicionNeta</t>
         </is>
       </c>
-      <c r="FD1" s="0" t="inlineStr">
+      <c r="FE1" t="inlineStr">
         <is>
           <t>valorCompradoNeto</t>
         </is>
       </c>
-      <c r="FE1" s="0" t="inlineStr">
+      <c r="FF1" t="inlineStr">
         <is>
           <t>valorInventarioNeto</t>
         </is>
       </c>
-      <c r="FF1" s="0" t="inlineStr">
+      <c r="FG1" t="inlineStr">
         <is>
           <t>cajaInicial</t>
         </is>
       </c>
-      <c r="FG1" s="0" t="inlineStr">
+      <c r="FH1" t="inlineStr">
         <is>
           <t>tasaNuevoPrestamo</t>
         </is>
       </c>
-      <c r="FH1" s="0" t="inlineStr">
+      <c r="FI1" t="inlineStr">
         <is>
           <t>interesMensual</t>
         </is>
       </c>
-      <c r="FI1" s="0" t="inlineStr">
+      <c r="FJ1" t="inlineStr">
         <is>
           <t>tasaMensual</t>
         </is>
       </c>
-      <c r="FJ1" s="0" t="inlineStr">
+      <c r="FK1" t="inlineStr">
         <is>
           <t>intereses</t>
         </is>
       </c>
-      <c r="FK1" s="0" t="inlineStr">
+      <c r="FL1" t="inlineStr">
         <is>
           <t>pagosOperacion</t>
         </is>
       </c>
-      <c r="FL1" s="0" t="inlineStr">
+      <c r="FM1" t="inlineStr">
         <is>
           <t>cajaFinal</t>
         </is>
       </c>
-      <c r="FM1" s="0" t="inlineStr">
+      <c r="FN1" t="inlineStr">
         <is>
           <t>depreciacionAcumulada</t>
         </is>
       </c>
-      <c r="FN1" s="0" t="inlineStr">
+      <c r="FO1" t="inlineStr">
         <is>
           <t>activosCosto</t>
         </is>
       </c>
-      <c r="FO1" s="0" t="inlineStr">
+      <c r="FP1" t="inlineStr">
         <is>
           <t>activosFijos</t>
         </is>
       </c>
-      <c r="FP1" s="0" t="inlineStr">
+      <c r="FQ1" t="inlineStr">
         <is>
           <t>financial.estadoResultados.ingresos</t>
         </is>
       </c>
-      <c r="FQ1" s="0" t="inlineStr">
+      <c r="FR1" t="inlineStr">
         <is>
           <t>financial.estadoResultados.ventasNetas</t>
         </is>
       </c>
-      <c r="FR1" s="0" t="inlineStr">
+      <c r="FS1" t="inlineStr">
         <is>
           <t>financial.estadoResultados.costos</t>
         </is>
       </c>
-      <c r="FS1" s="0" t="inlineStr">
+      <c r="FT1" t="inlineStr">
         <is>
           <t>financial.estadoResultados.utilidad</t>
         </is>
       </c>
-      <c r="FT1" s="0" t="inlineStr">
+      <c r="FU1" t="inlineStr">
         <is>
           <t>financial.estadoResultados.depreciacion</t>
         </is>
       </c>
-      <c r="FU1" s="0" t="inlineStr">
+      <c r="FV1" t="inlineStr">
         <is>
           <t>financial.estadoResultados.intereses</t>
         </is>
       </c>
-      <c r="FV1" s="0" t="inlineStr">
+      <c r="FW1" t="inlineStr">
         <is>
           <t>financial.estadoResultados.costosProduccion</t>
         </is>
       </c>
-      <c r="FW1" s="0" t="inlineStr">
+      <c r="FX1" t="inlineStr">
         <is>
           <t>financial.balanceCaja.cajaInicial</t>
         </is>
       </c>
-      <c r="FX1" s="0" t="inlineStr">
+      <c r="FY1" t="inlineStr">
         <is>
           <t>financial.balanceCaja.entradas</t>
         </is>
       </c>
-      <c r="FY1" s="0" t="inlineStr">
+      <c r="FZ1" t="inlineStr">
         <is>
           <t>financial.balanceCaja.salidas</t>
         </is>
       </c>
-      <c r="FZ1" s="0" t="inlineStr">
+      <c r="GA1" t="inlineStr">
         <is>
           <t>financial.balanceCaja.cajaFinal</t>
         </is>
       </c>
-      <c r="GA1" s="0" t="inlineStr">
+      <c r="GB1" t="inlineStr">
         <is>
           <t>financial.flujoCaja.cajaInicial</t>
         </is>
       </c>
-      <c r="GB1" s="0" t="inlineStr">
+      <c r="GC1" t="inlineStr">
         <is>
           <t>financial.flujoCaja.cobrosVentas</t>
         </is>
       </c>
-      <c r="GC1" s="0" t="inlineStr">
+      <c r="GD1" t="inlineStr">
         <is>
           <t>financial.flujoCaja.pagosOperacion</t>
         </is>
       </c>
-      <c r="GD1" s="0" t="inlineStr">
+      <c r="GE1" t="inlineStr">
         <is>
           <t>financial.flujoCaja.compraActivos</t>
         </is>
       </c>
-      <c r="GE1" s="0" t="inlineStr">
+      <c r="GF1" t="inlineStr">
         <is>
           <t>financial.flujoCaja.financiamiento</t>
         </is>
       </c>
-      <c r="GF1" s="0" t="inlineStr">
+      <c r="GG1" t="inlineStr">
         <is>
           <t>financial.flujoCaja.operacion</t>
         </is>
       </c>
-      <c r="GG1" s="0" t="inlineStr">
+      <c r="GH1" t="inlineStr">
         <is>
           <t>financial.flujoCaja.inversion</t>
         </is>
       </c>
-      <c r="GH1" s="0" t="inlineStr">
+      <c r="GI1" t="inlineStr">
         <is>
           <t>financial.flujoCaja.flujoNeto</t>
         </is>
       </c>
-      <c r="GI1" s="0" t="inlineStr">
+      <c r="GJ1" t="inlineStr">
         <is>
           <t>financial.flujoCaja.cajaFinal</t>
         </is>
       </c>
-      <c r="GJ1" s="0" t="inlineStr">
+      <c r="GK1" t="inlineStr">
         <is>
           <t>financial.balanceGeneral.efectivo</t>
         </is>
       </c>
-      <c r="GK1" s="0" t="inlineStr">
+      <c r="GL1" t="inlineStr">
         <is>
           <t>financial.balanceGeneral.activosFijos</t>
         </is>
       </c>
-      <c r="GL1" s="0" t="inlineStr">
+      <c r="GM1" t="inlineStr">
         <is>
           <t>financial.balanceGeneral.inventarioMP</t>
         </is>
       </c>
-      <c r="GM1" s="0" t="inlineStr">
+      <c r="GN1" t="inlineStr">
         <is>
           <t>financial.balanceGeneral.activos</t>
         </is>
       </c>
-      <c r="GN1" s="0" t="inlineStr">
+      <c r="GO1" t="inlineStr">
         <is>
           <t>financial.balanceGeneral.deuda</t>
         </is>
       </c>
-      <c r="GO1" s="0" t="inlineStr">
+      <c r="GP1" t="inlineStr">
         <is>
           <t>financial.balanceGeneral.patrimonio</t>
         </is>
       </c>
-      <c r="GP1" s="0" t="inlineStr">
+      <c r="GQ1" t="inlineStr">
         <is>
           <t>financial.balanceGeneral.pasivoPatrimonio</t>
         </is>
       </c>
-      <c r="GQ1" s="0" t="inlineStr">
+      <c r="GR1" t="inlineStr">
         <is>
           <t>financial.financiamiento.montoPrestamo</t>
         </is>
       </c>
-      <c r="GR1" s="0" t="inlineStr">
+      <c r="GS1" t="inlineStr">
         <is>
           <t>financial.financiamiento.tasaTEA</t>
         </is>
       </c>
-      <c r="GS1" s="0" t="inlineStr">
+      <c r="GT1" t="inlineStr">
         <is>
           <t>financial.financiamiento.deudaPrincipal</t>
         </is>
       </c>
-      <c r="GT1" s="0" t="inlineStr">
+      <c r="GU1" t="inlineStr">
         <is>
           <t>financial.financiamiento.tasaAdicionalProximoPrestamo</t>
         </is>
       </c>
-      <c r="GU1" s="0" t="inlineStr">
+      <c r="GV1" t="inlineStr">
         <is>
           <t>financial.financiamiento.tasaMensual</t>
         </is>
       </c>
-      <c r="GV1" s="0" t="inlineStr">
+      <c r="GW1" t="inlineStr">
         <is>
           <t>financial.financiamiento.intereses</t>
         </is>
@@ -5674,7 +5680,7 @@
         <v>0</v>
       </c>
       <c r="L2" s="0" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
       <c r="M2" s="0" t="inlineStr">
         <is>
@@ -5688,7 +5694,7 @@
       </c>
       <c r="O2" s="0" t="inlineStr">
         <is>
-          <t>INS-10A</t>
+          <t>COM-06B</t>
         </is>
       </c>
       <c r="P2" s="0" t="inlineStr">
@@ -6047,7 +6053,7 @@
         <v/>
       </c>
       <c r="DU2" s="0">
-        <f>(DB2*25+DD2*45+DF2*80+DI2*4+DK2*9+DN2*2+DP2*4+DR2*7)*0.8924</f>
+        <f>(DB2*25+DD2*45+DF2*80+DI2*4+DK2*9+DN2*2+DP2*4+DR2*7)*0.92</f>
         <v/>
       </c>
       <c r="DV2" s="0">
@@ -6121,246 +6127,249 @@
         <v/>
       </c>
       <c r="EN2" s="0">
-        <f>IFERROR(INDEX('Catalogo_Numerico_banca'!$G$2:$G$69,MATCH("",'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)*EJ2</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="EO2" s="0">
-        <f>(IFERROR(INDEX('Catalogo_Numerico_banca'!$G$2:$G$69,MATCH("INV-02A",'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0))*1</f>
+        <f>(0)*1</f>
         <v/>
       </c>
       <c r="EP2" s="0">
         <f>0</f>
         <v/>
       </c>
-      <c r="EQ2" s="0">
-        <f>DT2+DU2+DV2+DW2+L2+EL2+EM2+EN2+EO2+EP2</f>
-        <v/>
+      <c r="EQ2" s="0" t="n">
+        <v>0</v>
       </c>
       <c r="ER2" s="0">
-        <f>EK2-EQ2</f>
+        <f>DT2+DU2+DV2+DW2+L2+EL2+EM2+EN2+EO2+EP2+EQ2</f>
         <v/>
       </c>
       <c r="ES2" s="0">
+        <f>EK2-ER2</f>
+        <v/>
+      </c>
+      <c r="ET2" s="0">
         <f>AND(D2="SEG-03",AI2&lt;4,I2&gt;0)</f>
         <v/>
       </c>
-      <c r="ET2" s="0">
+      <c r="EU2" s="0">
         <f>AND(D2="SEG-03",AI2&gt;=7,I2&gt;0)</f>
         <v/>
       </c>
-      <c r="EU2" s="0">
+      <c r="EV2" s="0">
         <f>AF2&lt;4</f>
         <v/>
       </c>
-      <c r="EV2" s="0">
+      <c r="EW2" s="0">
         <f>AM2&gt;=2</f>
         <v/>
       </c>
-      <c r="EW2" s="0">
+      <c r="EX2" s="0">
         <f>AH2&lt;3</f>
         <v/>
       </c>
-      <c r="EX2" s="0">
+      <c r="EY2" s="0">
         <f>I2&gt;CE2</f>
         <v/>
       </c>
-      <c r="EY2" s="0">
+      <c r="EZ2" s="0">
         <f>CZ2&gt;EJ2</f>
         <v/>
       </c>
-      <c r="EZ2" s="0">
+      <c r="FA2" s="0">
         <f>AND(K2=0,AF2&lt;5)</f>
         <v/>
       </c>
-      <c r="FA2" s="0" t="n">
+      <c r="FB2" t="n">
         <v>1000000</v>
       </c>
-      <c r="FB2" s="0">
+      <c r="FC2">
         <f>1*2500*(1+0.03+0.02)+1*3500*(1+0.03+0.02)+1*1200*(1+0.03+0.02)+1*300*(1+0+0.01)</f>
         <v/>
       </c>
-      <c r="FC2" s="0">
+      <c r="FD2">
         <f>1*2500+1*3500+1*1200+1*300</f>
         <v/>
       </c>
-      <c r="FD2" s="0">
-        <f>(CF2*25+CH2*45+CJ2*80+CL2*4+CN2*9+CP2*2+CR2*4+CT2*7)*0.8924</f>
-        <v/>
-      </c>
-      <c r="FE2" s="0">
-        <f>(DC2*25+DE2*45+DG2*80+DJ2*4+DL2*9+DO2*2+DQ2*4+DS2*7)*0.8924</f>
-        <v/>
-      </c>
-      <c r="FF2" s="0">
-        <f>FA2</f>
-        <v/>
-      </c>
-      <c r="FG2" s="0">
+      <c r="FE2">
+        <f>(CF2*25+CH2*45+CJ2*80+CL2*4+CN2*9+CP2*2+CR2*4+CT2*7)*0.92</f>
+        <v/>
+      </c>
+      <c r="FF2">
+        <f>(DC2*25+DE2*45+DG2*80+DJ2*4+DL2*9+DO2*2+DQ2*4+DS2*7)*0.92</f>
+        <v/>
+      </c>
+      <c r="FG2">
+        <f>FB2</f>
+        <v/>
+      </c>
+      <c r="FH2">
         <f>(1+AR2/100)^(1/12)-1</f>
         <v/>
       </c>
-      <c r="FH2" s="0">
-        <f>0*0+AP2*FG2</f>
-        <v/>
-      </c>
-      <c r="FI2" s="0">
-        <f>IFERROR(FH2/(0+AP2),0)</f>
-        <v/>
-      </c>
-      <c r="FJ2" s="0">
-        <f>FH2*1</f>
-        <v/>
-      </c>
-      <c r="FK2" s="0">
-        <f>EQ2-DW2-DU2+FD2+FJ2</f>
-        <v/>
-      </c>
-      <c r="FL2" s="0">
-        <f>FF2+EK2+AP2-FK2-FB2</f>
-        <v/>
-      </c>
-      <c r="FM2" s="0">
+      <c r="FI2">
+        <f>0*0+AP2*FH2</f>
+        <v/>
+      </c>
+      <c r="FJ2">
+        <f>IFERROR(FI2/(0+AP2),0)</f>
+        <v/>
+      </c>
+      <c r="FK2">
+        <f>FI2*1</f>
+        <v/>
+      </c>
+      <c r="FL2">
+        <f>ER2-DW2-DU2+FE2+FK2</f>
+        <v/>
+      </c>
+      <c r="FM2">
+        <f>FG2+EK2+AP2-FL2-FC2</f>
+        <v/>
+      </c>
+      <c r="FN2">
         <f>0+DW2</f>
         <v/>
       </c>
-      <c r="FN2" s="0">
-        <f>0+FC2</f>
-        <v/>
-      </c>
-      <c r="FO2" s="0">
-        <f>FN2-FM2</f>
-        <v/>
-      </c>
-      <c r="FP2" s="0">
+      <c r="FO2">
+        <f>0+FD2</f>
+        <v/>
+      </c>
+      <c r="FP2">
+        <f>FO2-FN2</f>
+        <v/>
+      </c>
+      <c r="FQ2">
         <f>EK2</f>
         <v/>
       </c>
-      <c r="FQ2" s="0">
+      <c r="FR2">
         <f>EK2</f>
         <v/>
       </c>
-      <c r="FR2" s="0">
-        <f>EQ2+FJ2</f>
-        <v/>
-      </c>
-      <c r="FS2" s="0">
-        <f>ER2-FJ2</f>
-        <v/>
-      </c>
-      <c r="FT2" s="0">
+      <c r="FS2">
+        <f>ER2+FK2</f>
+        <v/>
+      </c>
+      <c r="FT2">
+        <f>ES2-FK2</f>
+        <v/>
+      </c>
+      <c r="FU2">
         <f>DW2</f>
         <v/>
       </c>
-      <c r="FU2" s="0">
+      <c r="FV2">
+        <f>FK2</f>
+        <v/>
+      </c>
+      <c r="FW2">
+        <f>ER2</f>
+        <v/>
+      </c>
+      <c r="FX2">
+        <f>FG2</f>
+        <v/>
+      </c>
+      <c r="FY2">
+        <f>EK2+AP2</f>
+        <v/>
+      </c>
+      <c r="FZ2">
+        <f>FL2+FC2</f>
+        <v/>
+      </c>
+      <c r="GA2">
+        <f>FM2</f>
+        <v/>
+      </c>
+      <c r="GB2">
+        <f>FG2</f>
+        <v/>
+      </c>
+      <c r="GC2">
+        <f>EK2</f>
+        <v/>
+      </c>
+      <c r="GD2">
+        <f>FL2</f>
+        <v/>
+      </c>
+      <c r="GE2">
+        <f>FC2</f>
+        <v/>
+      </c>
+      <c r="GF2">
+        <f>AP2</f>
+        <v/>
+      </c>
+      <c r="GG2">
+        <f>EK2-FL2</f>
+        <v/>
+      </c>
+      <c r="GH2">
+        <f>-FC2</f>
+        <v/>
+      </c>
+      <c r="GI2">
+        <f>FM2-FG2</f>
+        <v/>
+      </c>
+      <c r="GJ2">
+        <f>FM2</f>
+        <v/>
+      </c>
+      <c r="GK2">
+        <f>FM2</f>
+        <v/>
+      </c>
+      <c r="GL2">
+        <f>FP2</f>
+        <v/>
+      </c>
+      <c r="GM2">
+        <f>FF2</f>
+        <v/>
+      </c>
+      <c r="GN2">
+        <f>FM2+FP2+FF2</f>
+        <v/>
+      </c>
+      <c r="GO2">
+        <f>AS2</f>
+        <v/>
+      </c>
+      <c r="GP2">
+        <f>FM2+FP2+FF2-AS2</f>
+        <v/>
+      </c>
+      <c r="GQ2">
+        <f>FM2+FP2+FF2</f>
+        <v/>
+      </c>
+      <c r="GR2">
+        <f>AP2</f>
+        <v/>
+      </c>
+      <c r="GS2">
+        <f>AR2</f>
+        <v/>
+      </c>
+      <c r="GT2">
+        <f>AS2</f>
+        <v/>
+      </c>
+      <c r="GU2">
+        <f>AT2</f>
+        <v/>
+      </c>
+      <c r="GV2">
         <f>FJ2</f>
         <v/>
       </c>
-      <c r="FV2" s="0">
-        <f>EQ2</f>
-        <v/>
-      </c>
-      <c r="FW2" s="0">
-        <f>FF2</f>
-        <v/>
-      </c>
-      <c r="FX2" s="0">
-        <f>EK2+AP2</f>
-        <v/>
-      </c>
-      <c r="FY2" s="0">
-        <f>FK2+FB2</f>
-        <v/>
-      </c>
-      <c r="FZ2" s="0">
-        <f>FL2</f>
-        <v/>
-      </c>
-      <c r="GA2" s="0">
-        <f>FF2</f>
-        <v/>
-      </c>
-      <c r="GB2" s="0">
-        <f>EK2</f>
-        <v/>
-      </c>
-      <c r="GC2" s="0">
+      <c r="GW2">
         <f>FK2</f>
-        <v/>
-      </c>
-      <c r="GD2" s="0">
-        <f>FB2</f>
-        <v/>
-      </c>
-      <c r="GE2" s="0">
-        <f>AP2</f>
-        <v/>
-      </c>
-      <c r="GF2" s="0">
-        <f>EK2-FK2</f>
-        <v/>
-      </c>
-      <c r="GG2" s="0">
-        <f>-FB2</f>
-        <v/>
-      </c>
-      <c r="GH2" s="0">
-        <f>FL2-FF2</f>
-        <v/>
-      </c>
-      <c r="GI2" s="0">
-        <f>FL2</f>
-        <v/>
-      </c>
-      <c r="GJ2" s="0">
-        <f>FL2</f>
-        <v/>
-      </c>
-      <c r="GK2" s="0">
-        <f>FO2</f>
-        <v/>
-      </c>
-      <c r="GL2" s="0">
-        <f>FE2</f>
-        <v/>
-      </c>
-      <c r="GM2" s="0">
-        <f>FL2+FO2+FE2</f>
-        <v/>
-      </c>
-      <c r="GN2" s="0">
-        <f>AS2</f>
-        <v/>
-      </c>
-      <c r="GO2" s="0">
-        <f>FL2+FO2+FE2-AS2</f>
-        <v/>
-      </c>
-      <c r="GP2" s="0">
-        <f>FL2+FO2+FE2</f>
-        <v/>
-      </c>
-      <c r="GQ2" s="0">
-        <f>AP2</f>
-        <v/>
-      </c>
-      <c r="GR2" s="0">
-        <f>AR2</f>
-        <v/>
-      </c>
-      <c r="GS2" s="0">
-        <f>AS2</f>
-        <v/>
-      </c>
-      <c r="GT2" s="0">
-        <f>AT2</f>
-        <v/>
-      </c>
-      <c r="GU2" s="0">
-        <f>FI2</f>
-        <v/>
-      </c>
-      <c r="GV2" s="0">
-        <f>FJ2</f>
         <v/>
       </c>
     </row>
@@ -6432,44 +6441,20 @@
       </c>
       <c r="P3" s="0" t="inlineStr">
         <is>
-          <t>INS-09A</t>
+          <t>RH-10B</t>
         </is>
       </c>
       <c r="Q3" s="0" t="inlineStr">
         <is>
-          <t>INS-10B</t>
-        </is>
-      </c>
-      <c r="R3" s="0" t="inlineStr">
-        <is>
-          <t>INS-11C</t>
-        </is>
-      </c>
-      <c r="S3" s="0" t="inlineStr">
-        <is>
-          <t>RH-10B</t>
-        </is>
-      </c>
-      <c r="T3" s="0" t="inlineStr">
-        <is>
-          <t>FIN-02B</t>
-        </is>
-      </c>
-      <c r="U3" s="0" t="inlineStr">
-        <is>
-          <t>COM-06A</t>
-        </is>
-      </c>
-      <c r="V3" s="0" t="inlineStr">
-        <is>
-          <t>INF-11A</t>
-        </is>
-      </c>
-      <c r="W3" s="0" t="inlineStr">
-        <is>
-          <t>INS-12A</t>
-        </is>
-      </c>
+          <t>COM-06B</t>
+        </is>
+      </c>
+      <c r="R3" s="0" t="inlineStr"/>
+      <c r="S3" s="0" t="inlineStr"/>
+      <c r="T3" s="0" t="inlineStr"/>
+      <c r="U3" s="0" t="inlineStr"/>
+      <c r="V3" s="0" t="inlineStr"/>
+      <c r="W3" s="0" t="inlineStr"/>
       <c r="X3" s="0" t="inlineStr"/>
       <c r="Y3" s="0" t="inlineStr"/>
       <c r="Z3" s="0" t="inlineStr"/>
@@ -6479,15 +6464,15 @@
       <c r="AD3" s="0" t="inlineStr"/>
       <c r="AE3" s="0" t="inlineStr"/>
       <c r="AF3" s="0">
-        <f>IFERROR(INDEX('Catalogo_Numerico_banca'!$I$2:$I$69,MATCH(N3,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$I$2:$I$69,MATCH(O3,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$I$2:$I$69,MATCH(P3,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$I$2:$I$69,MATCH(Q3,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$I$2:$I$69,MATCH(R3,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$I$2:$I$69,MATCH(S3,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$I$2:$I$69,MATCH(T3,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$I$2:$I$69,MATCH(U3,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$I$2:$I$69,MATCH(V3,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$I$2:$I$69,MATCH(W3,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)</f>
+        <f>IFERROR(INDEX('Catalogo_Numerico_banca'!$I$2:$I$69,MATCH(N3,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$I$2:$I$69,MATCH(O3,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$I$2:$I$69,MATCH(P3,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$I$2:$I$69,MATCH(Q3,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)</f>
         <v/>
       </c>
       <c r="AG3" s="0">
-        <f>IFERROR(INDEX('Catalogo_Numerico_banca'!$J$2:$J$69,MATCH(N3,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$J$2:$J$69,MATCH(O3,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$J$2:$J$69,MATCH(P3,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$J$2:$J$69,MATCH(Q3,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$J$2:$J$69,MATCH(R3,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$J$2:$J$69,MATCH(S3,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$J$2:$J$69,MATCH(T3,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$J$2:$J$69,MATCH(U3,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$J$2:$J$69,MATCH(V3,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$J$2:$J$69,MATCH(W3,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)</f>
+        <f>IFERROR(INDEX('Catalogo_Numerico_banca'!$J$2:$J$69,MATCH(N3,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$J$2:$J$69,MATCH(O3,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$J$2:$J$69,MATCH(P3,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$J$2:$J$69,MATCH(Q3,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)</f>
         <v/>
       </c>
       <c r="AH3" s="0">
-        <f>IFERROR(INDEX('Catalogo_Numerico_banca'!$K$2:$K$69,MATCH(N3,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$K$2:$K$69,MATCH(O3,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$K$2:$K$69,MATCH(P3,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$K$2:$K$69,MATCH(Q3,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$K$2:$K$69,MATCH(R3,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$K$2:$K$69,MATCH(S3,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$K$2:$K$69,MATCH(T3,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$K$2:$K$69,MATCH(U3,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$K$2:$K$69,MATCH(V3,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$K$2:$K$69,MATCH(W3,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)</f>
+        <f>IFERROR(INDEX('Catalogo_Numerico_banca'!$K$2:$K$69,MATCH(N3,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$K$2:$K$69,MATCH(O3,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$K$2:$K$69,MATCH(P3,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$K$2:$K$69,MATCH(Q3,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)</f>
         <v/>
       </c>
       <c r="AI3" s="0">
@@ -6814,15 +6799,15 @@
         <v/>
       </c>
       <c r="DU3" s="0">
-        <f>(DB3*25+DD3*45+DF3*80+DI3*4+DK3*9+DN3*2+DP3*4+DR3*7)*0.9016000000000001</f>
+        <f>(DB3*25+DD3*45+DF3*80+DI3*4+DK3*9+DN3*2+DP3*4+DR3*7)*0.92</f>
         <v/>
       </c>
       <c r="DV3" s="0">
-        <f>1*2500*0.05/12*1+1*3500*0.05/12*1+1*1200*0.05/12*1+1*300*0.05/12*1+IFERROR(INDEX('Catalogo_Numerico_banca'!$G$2:$G$69,MATCH(V3,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)</f>
+        <f>1*2500*0.05/12*1+1*3500*0.05/12*1+1*1200*0.05/12*1+1*300*0.05/12*1</f>
         <v/>
       </c>
       <c r="DW3" s="0">
-        <f>1*(2375.0*CZ3/100000)+1*(3325.0*CZ3/100000)+1*(1140.0*CZ3/100000)+1*(285.0*CZ3/100000)</f>
+        <f>1*(2375.0/10/12*1)+1*(3325.0/10/12*1)+1*(1140.0/8/12*1)+1*(285.0/5/12*1)</f>
         <v/>
       </c>
       <c r="DX3" s="0">
@@ -6888,246 +6873,249 @@
         <v/>
       </c>
       <c r="EN3" s="0">
-        <f>IFERROR(INDEX('Catalogo_Numerico_banca'!$G$2:$G$69,MATCH("COM-06A",'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)*EJ3</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="EO3" s="0">
-        <f>(IFERROR(INDEX('Catalogo_Numerico_banca'!$G$2:$G$69,MATCH("COM-01A",'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$G$2:$G$69,MATCH("INS-12A",'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0))*1</f>
+        <f>(IFERROR(INDEX('Catalogo_Numerico_banca'!$G$2:$G$69,MATCH("COM-01A",'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0))*1</f>
         <v/>
       </c>
       <c r="EP3" s="0">
         <f>0</f>
         <v/>
       </c>
-      <c r="EQ3" s="0">
-        <f>DT3+DU3+DV3+DW3+L3+EL3+EM3+EN3+EO3+EP3</f>
-        <v/>
+      <c r="EQ3" s="0" t="n">
+        <v>0</v>
       </c>
       <c r="ER3" s="0">
-        <f>EK3-EQ3</f>
+        <f>DT3+DU3+DV3+DW3+L3+EL3+EM3+EN3+EO3+EP3+EQ3</f>
         <v/>
       </c>
       <c r="ES3" s="0">
+        <f>EK3-ER3</f>
+        <v/>
+      </c>
+      <c r="ET3" s="0">
         <f>AND(D3="SEG-03",AI3&lt;4,I3&gt;0)</f>
         <v/>
       </c>
-      <c r="ET3" s="0">
+      <c r="EU3" s="0">
         <f>AND(D3="SEG-03",AI3&gt;=7,I3&gt;0)</f>
         <v/>
       </c>
-      <c r="EU3" s="0">
+      <c r="EV3" s="0">
         <f>AF3&lt;4</f>
         <v/>
       </c>
-      <c r="EV3" s="0">
+      <c r="EW3" s="0">
         <f>AM3&gt;=2</f>
         <v/>
       </c>
-      <c r="EW3" s="0">
+      <c r="EX3" s="0">
         <f>AH3&lt;3</f>
         <v/>
       </c>
-      <c r="EX3" s="0">
+      <c r="EY3" s="0">
         <f>I3&gt;CE3</f>
         <v/>
       </c>
-      <c r="EY3" s="0">
+      <c r="EZ3" s="0">
         <f>CZ3&gt;EJ3</f>
         <v/>
       </c>
-      <c r="EZ3" s="0">
+      <c r="FA3" s="0">
         <f>AND(K3=0,AF3&lt;5)</f>
         <v/>
       </c>
-      <c r="FA3" s="0" t="n">
+      <c r="FB3" t="n">
         <v>1000000</v>
       </c>
-      <c r="FB3" s="0">
+      <c r="FC3">
         <f>0*2500*(1+0.03+0.02)+0*3500*(1+0.03+0.02)+0*1200*(1+0.03+0.02)+0*300*(1+0+0.01)</f>
         <v/>
       </c>
-      <c r="FC3" s="0">
+      <c r="FD3">
         <f>0*2500+0*3500+0*1200+0*300</f>
         <v/>
       </c>
-      <c r="FD3" s="0">
-        <f>(CF3*25+CH3*45+CJ3*80+CL3*4+CN3*9+CP3*2+CR3*4+CT3*7)*0.9016000000000001</f>
-        <v/>
-      </c>
-      <c r="FE3" s="0">
-        <f>(DC3*25+DE3*45+DG3*80+DJ3*4+DL3*9+DO3*2+DQ3*4+DS3*7)*0.9016000000000001</f>
-        <v/>
-      </c>
-      <c r="FF3" s="0">
-        <f>FL2</f>
-        <v/>
-      </c>
-      <c r="FG3" s="0">
+      <c r="FE3">
+        <f>(CF3*25+CH3*45+CJ3*80+CL3*4+CN3*9+CP3*2+CR3*4+CT3*7)*0.92</f>
+        <v/>
+      </c>
+      <c r="FF3">
+        <f>(DC3*25+DE3*45+DG3*80+DJ3*4+DL3*9+DO3*2+DQ3*4+DS3*7)*0.92</f>
+        <v/>
+      </c>
+      <c r="FG3">
+        <f>FM2</f>
+        <v/>
+      </c>
+      <c r="FH3">
         <f>(1+AR3/100)^(1/12)-1</f>
         <v/>
       </c>
-      <c r="FH3" s="0">
-        <f>AS2*FI2+AP3*FG3</f>
-        <v/>
-      </c>
-      <c r="FI3" s="0">
-        <f>IFERROR(FH3/(AS2+AP3),0)</f>
-        <v/>
-      </c>
-      <c r="FJ3" s="0">
-        <f>FH3*1</f>
-        <v/>
-      </c>
-      <c r="FK3" s="0">
-        <f>EQ3-DW3-DU3+FD3+FJ3</f>
-        <v/>
-      </c>
-      <c r="FL3" s="0">
-        <f>FF3+EK3+AP3-FK3-FB3</f>
-        <v/>
-      </c>
-      <c r="FM3" s="0">
-        <f>FM2+DW3</f>
-        <v/>
-      </c>
-      <c r="FN3" s="0">
-        <f>FN2+FC3</f>
-        <v/>
-      </c>
-      <c r="FO3" s="0">
-        <f>FN3-FM3</f>
-        <v/>
-      </c>
-      <c r="FP3" s="0">
+      <c r="FI3">
+        <f>AS2*FJ2+AP3*FH3</f>
+        <v/>
+      </c>
+      <c r="FJ3">
+        <f>IFERROR(FI3/(AS2+AP3),0)</f>
+        <v/>
+      </c>
+      <c r="FK3">
+        <f>FI3*1</f>
+        <v/>
+      </c>
+      <c r="FL3">
+        <f>ER3-DW3-DU3+FE3+FK3</f>
+        <v/>
+      </c>
+      <c r="FM3">
+        <f>FG3+EK3+AP3-FL3-FC3</f>
+        <v/>
+      </c>
+      <c r="FN3">
+        <f>FN2+DW3</f>
+        <v/>
+      </c>
+      <c r="FO3">
+        <f>FO2+FD3</f>
+        <v/>
+      </c>
+      <c r="FP3">
+        <f>FO3-FN3</f>
+        <v/>
+      </c>
+      <c r="FQ3">
         <f>EK3</f>
         <v/>
       </c>
-      <c r="FQ3" s="0">
+      <c r="FR3">
         <f>EK3</f>
         <v/>
       </c>
-      <c r="FR3" s="0">
-        <f>EQ3+FJ3</f>
-        <v/>
-      </c>
-      <c r="FS3" s="0">
-        <f>ER3-FJ3</f>
-        <v/>
-      </c>
-      <c r="FT3" s="0">
+      <c r="FS3">
+        <f>ER3+FK3</f>
+        <v/>
+      </c>
+      <c r="FT3">
+        <f>ES3-FK3</f>
+        <v/>
+      </c>
+      <c r="FU3">
         <f>DW3</f>
         <v/>
       </c>
-      <c r="FU3" s="0">
+      <c r="FV3">
+        <f>FK3</f>
+        <v/>
+      </c>
+      <c r="FW3">
+        <f>ER3</f>
+        <v/>
+      </c>
+      <c r="FX3">
+        <f>FG3</f>
+        <v/>
+      </c>
+      <c r="FY3">
+        <f>EK3+AP3</f>
+        <v/>
+      </c>
+      <c r="FZ3">
+        <f>FL3+FC3</f>
+        <v/>
+      </c>
+      <c r="GA3">
+        <f>FM3</f>
+        <v/>
+      </c>
+      <c r="GB3">
+        <f>FG3</f>
+        <v/>
+      </c>
+      <c r="GC3">
+        <f>EK3</f>
+        <v/>
+      </c>
+      <c r="GD3">
+        <f>FL3</f>
+        <v/>
+      </c>
+      <c r="GE3">
+        <f>FC3</f>
+        <v/>
+      </c>
+      <c r="GF3">
+        <f>AP3</f>
+        <v/>
+      </c>
+      <c r="GG3">
+        <f>EK3-FL3</f>
+        <v/>
+      </c>
+      <c r="GH3">
+        <f>-FC3</f>
+        <v/>
+      </c>
+      <c r="GI3">
+        <f>FM3-FG3</f>
+        <v/>
+      </c>
+      <c r="GJ3">
+        <f>FM3</f>
+        <v/>
+      </c>
+      <c r="GK3">
+        <f>FM3</f>
+        <v/>
+      </c>
+      <c r="GL3">
+        <f>FP3</f>
+        <v/>
+      </c>
+      <c r="GM3">
+        <f>FF3</f>
+        <v/>
+      </c>
+      <c r="GN3">
+        <f>FM3+FP3+FF3</f>
+        <v/>
+      </c>
+      <c r="GO3">
+        <f>AS3</f>
+        <v/>
+      </c>
+      <c r="GP3">
+        <f>FM3+FP3+FF3-AS3</f>
+        <v/>
+      </c>
+      <c r="GQ3">
+        <f>FM3+FP3+FF3</f>
+        <v/>
+      </c>
+      <c r="GR3">
+        <f>AP3</f>
+        <v/>
+      </c>
+      <c r="GS3">
+        <f>AR3</f>
+        <v/>
+      </c>
+      <c r="GT3">
+        <f>AS3</f>
+        <v/>
+      </c>
+      <c r="GU3">
+        <f>AT3</f>
+        <v/>
+      </c>
+      <c r="GV3">
         <f>FJ3</f>
         <v/>
       </c>
-      <c r="FV3" s="0">
-        <f>EQ3</f>
-        <v/>
-      </c>
-      <c r="FW3" s="0">
-        <f>FF3</f>
-        <v/>
-      </c>
-      <c r="FX3" s="0">
-        <f>EK3+AP3</f>
-        <v/>
-      </c>
-      <c r="FY3" s="0">
-        <f>FK3+FB3</f>
-        <v/>
-      </c>
-      <c r="FZ3" s="0">
-        <f>FL3</f>
-        <v/>
-      </c>
-      <c r="GA3" s="0">
-        <f>FF3</f>
-        <v/>
-      </c>
-      <c r="GB3" s="0">
-        <f>EK3</f>
-        <v/>
-      </c>
-      <c r="GC3" s="0">
+      <c r="GW3">
         <f>FK3</f>
-        <v/>
-      </c>
-      <c r="GD3" s="0">
-        <f>FB3</f>
-        <v/>
-      </c>
-      <c r="GE3" s="0">
-        <f>AP3</f>
-        <v/>
-      </c>
-      <c r="GF3" s="0">
-        <f>EK3-FK3</f>
-        <v/>
-      </c>
-      <c r="GG3" s="0">
-        <f>-FB3</f>
-        <v/>
-      </c>
-      <c r="GH3" s="0">
-        <f>FL3-FF3</f>
-        <v/>
-      </c>
-      <c r="GI3" s="0">
-        <f>FL3</f>
-        <v/>
-      </c>
-      <c r="GJ3" s="0">
-        <f>FL3</f>
-        <v/>
-      </c>
-      <c r="GK3" s="0">
-        <f>FO3</f>
-        <v/>
-      </c>
-      <c r="GL3" s="0">
-        <f>FE3</f>
-        <v/>
-      </c>
-      <c r="GM3" s="0">
-        <f>FL3+FO3+FE3</f>
-        <v/>
-      </c>
-      <c r="GN3" s="0">
-        <f>AS3</f>
-        <v/>
-      </c>
-      <c r="GO3" s="0">
-        <f>FL3+FO3+FE3-AS3</f>
-        <v/>
-      </c>
-      <c r="GP3" s="0">
-        <f>FL3+FO3+FE3</f>
-        <v/>
-      </c>
-      <c r="GQ3" s="0">
-        <f>AP3</f>
-        <v/>
-      </c>
-      <c r="GR3" s="0">
-        <f>AR3</f>
-        <v/>
-      </c>
-      <c r="GS3" s="0">
-        <f>AS3</f>
-        <v/>
-      </c>
-      <c r="GT3" s="0">
-        <f>AT3</f>
-        <v/>
-      </c>
-      <c r="GU3" s="0">
-        <f>FI3</f>
-        <v/>
-      </c>
-      <c r="GV3" s="0">
-        <f>FJ3</f>
         <v/>
       </c>
     </row>
@@ -7194,49 +7182,25 @@
       </c>
       <c r="O4" s="0" t="inlineStr">
         <is>
-          <t>INS-09A</t>
+          <t>RH-10B</t>
         </is>
       </c>
       <c r="P4" s="0" t="inlineStr">
         <is>
-          <t>INS-10B</t>
+          <t>COM-06B</t>
         </is>
       </c>
       <c r="Q4" s="0" t="inlineStr">
         <is>
-          <t>INS-11C</t>
-        </is>
-      </c>
-      <c r="R4" s="0" t="inlineStr">
-        <is>
-          <t>RH-10B</t>
-        </is>
-      </c>
-      <c r="S4" s="0" t="inlineStr">
-        <is>
-          <t>FIN-02B</t>
-        </is>
-      </c>
-      <c r="T4" s="0" t="inlineStr">
-        <is>
-          <t>COM-06A</t>
-        </is>
-      </c>
-      <c r="U4" s="0" t="inlineStr">
-        <is>
-          <t>INF-11A</t>
-        </is>
-      </c>
-      <c r="V4" s="0" t="inlineStr">
-        <is>
-          <t>INS-12A</t>
-        </is>
-      </c>
-      <c r="W4" s="0" t="inlineStr">
-        <is>
           <t>FIN-01A</t>
         </is>
       </c>
+      <c r="R4" s="0" t="inlineStr"/>
+      <c r="S4" s="0" t="inlineStr"/>
+      <c r="T4" s="0" t="inlineStr"/>
+      <c r="U4" s="0" t="inlineStr"/>
+      <c r="V4" s="0" t="inlineStr"/>
+      <c r="W4" s="0" t="inlineStr"/>
       <c r="X4" s="0" t="inlineStr"/>
       <c r="Y4" s="0" t="inlineStr"/>
       <c r="Z4" s="0" t="inlineStr"/>
@@ -7246,15 +7210,15 @@
       <c r="AD4" s="0" t="inlineStr"/>
       <c r="AE4" s="0" t="inlineStr"/>
       <c r="AF4" s="0">
-        <f>IFERROR(INDEX('Catalogo_Numerico_banca'!$I$2:$I$69,MATCH(N4,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$I$2:$I$69,MATCH(O4,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$I$2:$I$69,MATCH(P4,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$I$2:$I$69,MATCH(Q4,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$I$2:$I$69,MATCH(R4,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$I$2:$I$69,MATCH(S4,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$I$2:$I$69,MATCH(T4,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$I$2:$I$69,MATCH(U4,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$I$2:$I$69,MATCH(V4,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$I$2:$I$69,MATCH(W4,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)</f>
+        <f>IFERROR(INDEX('Catalogo_Numerico_banca'!$I$2:$I$69,MATCH(N4,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$I$2:$I$69,MATCH(O4,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$I$2:$I$69,MATCH(P4,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$I$2:$I$69,MATCH(Q4,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)</f>
         <v/>
       </c>
       <c r="AG4" s="0">
-        <f>IFERROR(INDEX('Catalogo_Numerico_banca'!$J$2:$J$69,MATCH(N4,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$J$2:$J$69,MATCH(O4,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$J$2:$J$69,MATCH(P4,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$J$2:$J$69,MATCH(Q4,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$J$2:$J$69,MATCH(R4,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$J$2:$J$69,MATCH(S4,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$J$2:$J$69,MATCH(T4,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$J$2:$J$69,MATCH(U4,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$J$2:$J$69,MATCH(V4,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$J$2:$J$69,MATCH(W4,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)</f>
+        <f>IFERROR(INDEX('Catalogo_Numerico_banca'!$J$2:$J$69,MATCH(N4,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$J$2:$J$69,MATCH(O4,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$J$2:$J$69,MATCH(P4,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$J$2:$J$69,MATCH(Q4,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)</f>
         <v/>
       </c>
       <c r="AH4" s="0">
-        <f>IFERROR(INDEX('Catalogo_Numerico_banca'!$K$2:$K$69,MATCH(N4,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$K$2:$K$69,MATCH(O4,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$K$2:$K$69,MATCH(P4,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$K$2:$K$69,MATCH(Q4,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$K$2:$K$69,MATCH(R4,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$K$2:$K$69,MATCH(S4,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$K$2:$K$69,MATCH(T4,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$K$2:$K$69,MATCH(U4,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$K$2:$K$69,MATCH(V4,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$K$2:$K$69,MATCH(W4,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)</f>
+        <f>IFERROR(INDEX('Catalogo_Numerico_banca'!$K$2:$K$69,MATCH(N4,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$K$2:$K$69,MATCH(O4,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$K$2:$K$69,MATCH(P4,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$K$2:$K$69,MATCH(Q4,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)</f>
         <v/>
       </c>
       <c r="AI4" s="0">
@@ -7581,15 +7545,15 @@
         <v/>
       </c>
       <c r="DU4" s="0">
-        <f>(DB4*25+DD4*45+DF4*80+DI4*4+DK4*9+DN4*2+DP4*4+DR4*7)*0.9016000000000001</f>
+        <f>(DB4*25+DD4*45+DF4*80+DI4*4+DK4*9+DN4*2+DP4*4+DR4*7)*0.92</f>
         <v/>
       </c>
       <c r="DV4" s="0">
-        <f>1*2500*0.05/12*1+1*3500*0.05/12*1+1*1200*0.05/12*1+1*300*0.05/12*1+IFERROR(INDEX('Catalogo_Numerico_banca'!$G$2:$G$69,MATCH(U4,'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)</f>
+        <f>1*2500*0.05/12*1+1*3500*0.05/12*1+1*1200*0.05/12*1+1*300*0.05/12*1</f>
         <v/>
       </c>
       <c r="DW4" s="0">
-        <f>1*(2375.0*CZ4/100000)+1*(3325.0*CZ4/100000)+1*(1140.0*CZ4/100000)+1*(285.0*CZ4/100000)</f>
+        <f>1*(2375.0/10/12*1)+1*(3325.0/10/12*1)+1*(1140.0/8/12*1)+1*(285.0/5/12*1)</f>
         <v/>
       </c>
       <c r="DX4" s="0">
@@ -7655,246 +7619,249 @@
         <v/>
       </c>
       <c r="EN4" s="0">
-        <f>IFERROR(INDEX('Catalogo_Numerico_banca'!$G$2:$G$69,MATCH("COM-06A",'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)*EJ4</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="EO4" s="0">
-        <f>(IFERROR(INDEX('Catalogo_Numerico_banca'!$G$2:$G$69,MATCH("COM-01A",'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_banca'!$G$2:$G$69,MATCH("INS-12A",'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0))*1</f>
+        <f>(IFERROR(INDEX('Catalogo_Numerico_banca'!$G$2:$G$69,MATCH("COM-01A",'Catalogo_Numerico_banca'!$A$2:$A$69,0)),0))*1</f>
         <v/>
       </c>
       <c r="EP4" s="0">
         <f>0</f>
         <v/>
       </c>
-      <c r="EQ4" s="0">
-        <f>DT4+DU4+DV4+DW4+L4+EL4+EM4+EN4+EO4+EP4</f>
-        <v/>
+      <c r="EQ4" s="0" t="n">
+        <v>0</v>
       </c>
       <c r="ER4" s="0">
-        <f>EK4-EQ4</f>
+        <f>DT4+DU4+DV4+DW4+L4+EL4+EM4+EN4+EO4+EP4+EQ4</f>
         <v/>
       </c>
       <c r="ES4" s="0">
+        <f>EK4-ER4</f>
+        <v/>
+      </c>
+      <c r="ET4" s="0">
         <f>AND(D4="SEG-03",AI4&lt;4,I4&gt;0)</f>
         <v/>
       </c>
-      <c r="ET4" s="0">
+      <c r="EU4" s="0">
         <f>AND(D4="SEG-03",AI4&gt;=7,I4&gt;0)</f>
         <v/>
       </c>
-      <c r="EU4" s="0">
+      <c r="EV4" s="0">
         <f>AF4&lt;4</f>
         <v/>
       </c>
-      <c r="EV4" s="0">
+      <c r="EW4" s="0">
         <f>AM4&gt;=2</f>
         <v/>
       </c>
-      <c r="EW4" s="0">
+      <c r="EX4" s="0">
         <f>AH4&lt;3</f>
         <v/>
       </c>
-      <c r="EX4" s="0">
+      <c r="EY4" s="0">
         <f>I4&gt;CE4</f>
         <v/>
       </c>
-      <c r="EY4" s="0">
+      <c r="EZ4" s="0">
         <f>CZ4&gt;EJ4</f>
         <v/>
       </c>
-      <c r="EZ4" s="0">
+      <c r="FA4" s="0">
         <f>AND(K4=0,AF4&lt;5)</f>
         <v/>
       </c>
-      <c r="FA4" s="0" t="n">
+      <c r="FB4" t="n">
         <v>1000000</v>
       </c>
-      <c r="FB4" s="0">
+      <c r="FC4">
         <f>0*2500*(1+0.03+0.02)+0*3500*(1+0.03+0.02)+0*1200*(1+0.03+0.02)+0*300*(1+0+0.01)</f>
         <v/>
       </c>
-      <c r="FC4" s="0">
+      <c r="FD4">
         <f>0*2500+0*3500+0*1200+0*300</f>
         <v/>
       </c>
-      <c r="FD4" s="0">
-        <f>(CF4*25+CH4*45+CJ4*80+CL4*4+CN4*9+CP4*2+CR4*4+CT4*7)*0.9016000000000001</f>
-        <v/>
-      </c>
-      <c r="FE4" s="0">
-        <f>(DC4*25+DE4*45+DG4*80+DJ4*4+DL4*9+DO4*2+DQ4*4+DS4*7)*0.9016000000000001</f>
-        <v/>
-      </c>
-      <c r="FF4" s="0">
-        <f>FL3</f>
-        <v/>
-      </c>
-      <c r="FG4" s="0">
+      <c r="FE4">
+        <f>(CF4*25+CH4*45+CJ4*80+CL4*4+CN4*9+CP4*2+CR4*4+CT4*7)*0.92</f>
+        <v/>
+      </c>
+      <c r="FF4">
+        <f>(DC4*25+DE4*45+DG4*80+DJ4*4+DL4*9+DO4*2+DQ4*4+DS4*7)*0.92</f>
+        <v/>
+      </c>
+      <c r="FG4">
+        <f>FM3</f>
+        <v/>
+      </c>
+      <c r="FH4">
         <f>(1+AR4/100)^(1/12)-1</f>
         <v/>
       </c>
-      <c r="FH4" s="0">
-        <f>AS3*FI3+AP4*FG4</f>
-        <v/>
-      </c>
-      <c r="FI4" s="0">
-        <f>IFERROR(FH4/(AS3+AP4),0)</f>
-        <v/>
-      </c>
-      <c r="FJ4" s="0">
-        <f>FH4*1</f>
-        <v/>
-      </c>
-      <c r="FK4" s="0">
-        <f>EQ4-DW4-DU4+FD4+FJ4</f>
-        <v/>
-      </c>
-      <c r="FL4" s="0">
-        <f>FF4+EK4+AP4-FK4-FB4</f>
-        <v/>
-      </c>
-      <c r="FM4" s="0">
-        <f>FM3+DW4</f>
-        <v/>
-      </c>
-      <c r="FN4" s="0">
-        <f>FN3+FC4</f>
-        <v/>
-      </c>
-      <c r="FO4" s="0">
-        <f>FN4-FM4</f>
-        <v/>
-      </c>
-      <c r="FP4" s="0">
+      <c r="FI4">
+        <f>AS3*FJ3+AP4*FH4</f>
+        <v/>
+      </c>
+      <c r="FJ4">
+        <f>IFERROR(FI4/(AS3+AP4),0)</f>
+        <v/>
+      </c>
+      <c r="FK4">
+        <f>FI4*1</f>
+        <v/>
+      </c>
+      <c r="FL4">
+        <f>ER4-DW4-DU4+FE4+FK4</f>
+        <v/>
+      </c>
+      <c r="FM4">
+        <f>FG4+EK4+AP4-FL4-FC4</f>
+        <v/>
+      </c>
+      <c r="FN4">
+        <f>FN3+DW4</f>
+        <v/>
+      </c>
+      <c r="FO4">
+        <f>FO3+FD4</f>
+        <v/>
+      </c>
+      <c r="FP4">
+        <f>FO4-FN4</f>
+        <v/>
+      </c>
+      <c r="FQ4">
         <f>EK4</f>
         <v/>
       </c>
-      <c r="FQ4" s="0">
+      <c r="FR4">
         <f>EK4</f>
         <v/>
       </c>
-      <c r="FR4" s="0">
-        <f>EQ4+FJ4</f>
-        <v/>
-      </c>
-      <c r="FS4" s="0">
-        <f>ER4-FJ4</f>
-        <v/>
-      </c>
-      <c r="FT4" s="0">
+      <c r="FS4">
+        <f>ER4+FK4</f>
+        <v/>
+      </c>
+      <c r="FT4">
+        <f>ES4-FK4</f>
+        <v/>
+      </c>
+      <c r="FU4">
         <f>DW4</f>
         <v/>
       </c>
-      <c r="FU4" s="0">
+      <c r="FV4">
+        <f>FK4</f>
+        <v/>
+      </c>
+      <c r="FW4">
+        <f>ER4</f>
+        <v/>
+      </c>
+      <c r="FX4">
+        <f>FG4</f>
+        <v/>
+      </c>
+      <c r="FY4">
+        <f>EK4+AP4</f>
+        <v/>
+      </c>
+      <c r="FZ4">
+        <f>FL4+FC4</f>
+        <v/>
+      </c>
+      <c r="GA4">
+        <f>FM4</f>
+        <v/>
+      </c>
+      <c r="GB4">
+        <f>FG4</f>
+        <v/>
+      </c>
+      <c r="GC4">
+        <f>EK4</f>
+        <v/>
+      </c>
+      <c r="GD4">
+        <f>FL4</f>
+        <v/>
+      </c>
+      <c r="GE4">
+        <f>FC4</f>
+        <v/>
+      </c>
+      <c r="GF4">
+        <f>AP4</f>
+        <v/>
+      </c>
+      <c r="GG4">
+        <f>EK4-FL4</f>
+        <v/>
+      </c>
+      <c r="GH4">
+        <f>-FC4</f>
+        <v/>
+      </c>
+      <c r="GI4">
+        <f>FM4-FG4</f>
+        <v/>
+      </c>
+      <c r="GJ4">
+        <f>FM4</f>
+        <v/>
+      </c>
+      <c r="GK4">
+        <f>FM4</f>
+        <v/>
+      </c>
+      <c r="GL4">
+        <f>FP4</f>
+        <v/>
+      </c>
+      <c r="GM4">
+        <f>FF4</f>
+        <v/>
+      </c>
+      <c r="GN4">
+        <f>FM4+FP4+FF4</f>
+        <v/>
+      </c>
+      <c r="GO4">
+        <f>AS4</f>
+        <v/>
+      </c>
+      <c r="GP4">
+        <f>FM4+FP4+FF4-AS4</f>
+        <v/>
+      </c>
+      <c r="GQ4">
+        <f>FM4+FP4+FF4</f>
+        <v/>
+      </c>
+      <c r="GR4">
+        <f>AP4</f>
+        <v/>
+      </c>
+      <c r="GS4">
+        <f>AR4</f>
+        <v/>
+      </c>
+      <c r="GT4">
+        <f>AS4</f>
+        <v/>
+      </c>
+      <c r="GU4">
+        <f>AT4</f>
+        <v/>
+      </c>
+      <c r="GV4">
         <f>FJ4</f>
         <v/>
       </c>
-      <c r="FV4" s="0">
-        <f>EQ4</f>
-        <v/>
-      </c>
-      <c r="FW4" s="0">
-        <f>FF4</f>
-        <v/>
-      </c>
-      <c r="FX4" s="0">
-        <f>EK4+AP4</f>
-        <v/>
-      </c>
-      <c r="FY4" s="0">
-        <f>FK4+FB4</f>
-        <v/>
-      </c>
-      <c r="FZ4" s="0">
-        <f>FL4</f>
-        <v/>
-      </c>
-      <c r="GA4" s="0">
-        <f>FF4</f>
-        <v/>
-      </c>
-      <c r="GB4" s="0">
-        <f>EK4</f>
-        <v/>
-      </c>
-      <c r="GC4" s="0">
+      <c r="GW4">
         <f>FK4</f>
-        <v/>
-      </c>
-      <c r="GD4" s="0">
-        <f>FB4</f>
-        <v/>
-      </c>
-      <c r="GE4" s="0">
-        <f>AP4</f>
-        <v/>
-      </c>
-      <c r="GF4" s="0">
-        <f>EK4-FK4</f>
-        <v/>
-      </c>
-      <c r="GG4" s="0">
-        <f>-FB4</f>
-        <v/>
-      </c>
-      <c r="GH4" s="0">
-        <f>FL4-FF4</f>
-        <v/>
-      </c>
-      <c r="GI4" s="0">
-        <f>FL4</f>
-        <v/>
-      </c>
-      <c r="GJ4" s="0">
-        <f>FL4</f>
-        <v/>
-      </c>
-      <c r="GK4" s="0">
-        <f>FO4</f>
-        <v/>
-      </c>
-      <c r="GL4" s="0">
-        <f>FE4</f>
-        <v/>
-      </c>
-      <c r="GM4" s="0">
-        <f>FL4+FO4+FE4</f>
-        <v/>
-      </c>
-      <c r="GN4" s="0">
-        <f>AS4</f>
-        <v/>
-      </c>
-      <c r="GO4" s="0">
-        <f>FL4+FO4+FE4-AS4</f>
-        <v/>
-      </c>
-      <c r="GP4" s="0">
-        <f>FL4+FO4+FE4</f>
-        <v/>
-      </c>
-      <c r="GQ4" s="0">
-        <f>AP4</f>
-        <v/>
-      </c>
-      <c r="GR4" s="0">
-        <f>AR4</f>
-        <v/>
-      </c>
-      <c r="GS4" s="0">
-        <f>AS4</f>
-        <v/>
-      </c>
-      <c r="GT4" s="0">
-        <f>AT4</f>
-        <v/>
-      </c>
-      <c r="GU4" s="0">
-        <f>FI4</f>
-        <v/>
-      </c>
-      <c r="GV4" s="0">
-        <f>FJ4</f>
         <v/>
       </c>
     </row>

</xml_diff>